<commit_message>
Blinder statt Blitz bei BlingBling (Kids, Maniac), Blinder hinter dem Titel-Lauftext
- Kids "chorus intro" und Maniac "rock intro": transition flash durch einen halb starken
  warmweißen Blinder (1 Beat) ersetzt. progFastBlingBling setzt die Helligkeit auf 255,
  der weiße Blitz zog auf der Matrix über 3,6 A. Timing und MIDI unverändert.
- Neu fxBlinderBehind(): Blinder füllt nur die dunklen LEDs (hinter dem Bild).
  songgen.py: blinder title: true meldet ihn im Titel-Lauftext-case der Scroll-Geräte an
  (Maniac Takt 12). Ohne title gleicher Code wie vorher.
- Demo 92 Part 71, Doku (LED-Effekte, Katalog, Skill-Regel gegen Blitz + BlingBling,
  FX-Pipeline-Plan, CLAUDE.md, README).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/songs/Kids_v1/quelle/struktur.xlsx
+++ b/songs/Kids_v1/quelle/struktur.xlsx
@@ -1174,8 +1174,8 @@
       <c r="C55" s="6" t="inlineStr">
         <is>
           <t>progFastBlingBling(15000, 8, 5), Farben SCHEME_NEON
-Ausgabe: Übergang flash 469 ms
-Weißer Blitz auf den Band-Einsatz, danach schnelle bunte Einzelblitze (wie bisher).</t>
+Ausgabe: Blinder bei 0 ms, 469 ms lang
+Warmweißer Blinder auf den Band-Einsatz (halbe Stärke, 1 Beat), danach schnelle bunte Einzelblitze (wie bisher).</t>
         </is>
       </c>
       <c r="D55" s="6" t="n"/>

</xml_diff>